<commit_message>
Update supplier tracker: FFT meeting held + scope changes sent
FFT (Germany) status EMAIL SENT -> MET. Recorded the post-meeting
follow-up: test specification + 3D CAD sent, and the scope changes
(hipot+functional merged into one module; power separated from
control/IO; semi-automated product-to-pallet connection; visual
inspection limited to HMI verification). Medium Drives scope to follow.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XCyDZxfZxZ3SBQAJkRpEXx
</commit_message>
<xml_diff>
--- a/SUPPLIERS/SUPPLIERS.xlsx
+++ b/SUPPLIERS/SUPPLIERS.xlsx
@@ -1123,20 +1123,25 @@
           <t>FFT Produktionssysteme</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Edgar Vöhringer (Account Manager)</t>
+        </is>
+      </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>info@fft.de</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>EMAIL SENT</t>
+          <t>info@fft.de
+Edgar Vöhringer &lt;edgar.voehringer@fft.de&gt;</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>MET</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>24/06/2026</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1146,12 +1151,12 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Waiting for reply</t>
+          <t>Sent test specification + 3D CAD and scope changes (26/06/2026). Medium Drives scope to follow this week. Next: await FFT feedback / schedule follow-up call.</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Email sent.</t>
+          <t>Fulda, Germany (Edgar Vöhringer). INBOUND contact. Meeting held 24/06/2026. Scope changes communicated: (1) Hipot + Functional tests merged into a SINGLE module; (2) Power connection separated from Control/IO - hipot uses only power connections, functional uses power + control; (3) Semi-automated product-to-pallet connection (busbars/needles/pogo - method TBD by supplier), connection movement &amp; fixturing by operator; (4) Visual inspection limited to verifying the HMI is working correctly. Test specification + 3D CAD sent. Medium Drives scope (higher power/current/size) to be sent this week.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update SUPPLIERS.xlsx: mark Comau as declined (23/06); refresh header date
</commit_message>
<xml_diff>
--- a/SUPPLIERS/SUPPLIERS.xlsx
+++ b/SUPPLIERS/SUPPLIERS.xlsx
@@ -653,7 +653,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>MODULAR ALL DRIVES - Supplier Contact Tracker  |  Aluizio Kleine / Industrial Engineering / WEG Drives and Controls  |  Updated: 26/06/2026</t>
+          <t>MODULAR ALL DRIVES - Supplier Contact Tracker  |  Aluizio Kleine / Industrial Engineering / WEG Drives and Controls  |  Updated: 30/06/2026</t>
         </is>
       </c>
     </row>
@@ -1016,11 +1016,13 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>MET</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="n">
-        <v>46332</v>
+          <t>DECLINED</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
@@ -1029,12 +1031,12 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Waiting for quotation</t>
+          <t>OUT - Declined 23/06/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Large automotive machine builder. Brazil presence (Betim/MG). PE-owned (One Equity Partners).</t>
+          <t>DECLINED (23/06/2026, Carla Cristina Haddad, Sales Coordinator - carla.cristina@comau.com): Unavailability of qualified workforce to absorb responsibilities beyond current and planned ones; high competitiveness required for this specific activity; challenging deadlines. Reiterated strong interest in future opportunities and remains open to new contacts that better fit Comau's resource allocation and expertise. Large automotive machine builder. Brazil presence (Betim/MG). PE-owned (One Equity Partners).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct supplier tracker per Aluizio's status review (02/07)
- Bosch, Autec, Mondragon, DMC, PIA: confirmed waiting for quotation
- MASMEC, BBS: quote received, pricing meeting scheduled to negotiate
  a reduction (date TBC)
- FFT: corrected to reflect Q&A answers + documents still pending to
  send (not already sent)
- Comau, Develop LLC, Tamadic, JR Automation: confirmed declined/
  disqualified (no change needed, already correct)
- Added action for all active suppliers: send updated Small-line
  scope + send Medium-line scope for quoting

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XCyDZxfZxZ3SBQAJkRpEXx
</commit_message>
<xml_diff>
--- a/SUPPLIERS/SUPPLIERS.xlsx
+++ b/SUPPLIERS/SUPPLIERS.xlsx
@@ -653,7 +653,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>MODULAR ALL DRIVES - Supplier Contact Tracker  |  Aluizio Kleine / Industrial Engineering / WEG Drives and Controls  |  Updated: 01/07/2026</t>
+          <t>MODULAR ALL DRIVES - Supplier Contact Tracker  |  Aluizio Kleine / Industrial Engineering / WEG Drives and Controls  |  Updated: 02/07/2026</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Waiting for WEG docs: test prescriptions + product dimensions table + terminal drawings</t>
+          <t>Waiting for quotation. WEG to send: test prescriptions + product dimensions table + terminal drawings. Send updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Waiting for quotation</t>
+          <t>Waiting for quotation. WEG to send: updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Waiting for quotation</t>
+          <t>Waiting for quotation. WEG to send: updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -991,12 +991,12 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Waiting for quotation. WEG to send: test prescription per module + confirm WEG PLC (not Siemens)</t>
+          <t>Quote C610222-1 received. Meeting scheduled to discuss the quote and negotiate price reduction. WEG to send: test prescription per module + confirm WEG PLC (not Siemens). Send updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Bari, Italy. Direct experience testing automotive inverters (hipot, functional, load). Bosch Rexroth TS2 conveyor. Brazil installs. All machines made in Italy. Digital twin w/ Plant Simulation.</t>
+          <t>Bari, Italy. Direct experience testing automotive inverters (hipot, functional, load). Bosch Rexroth TS2 conveyor. Brazil installs. All machines made in Italy. Digital twin w/ Plant Simulation. Meeting scheduled (date TBC) to review pricing.</t>
         </is>
       </c>
     </row>
@@ -1153,12 +1153,12 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Sent test specification + 3D CAD and scope changes (26/06/2026). Medium Drives scope to follow this week. Next: await FFT feedback / schedule follow-up call.</t>
+          <t>WEG to answer FFT's 6 technical questions and send the WEG inverter programming reference doc + product CAD. Send updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Fulda, Germany (Edgar Vöhringer). INBOUND contact. Meeting held 24/06/2026. Scope changes communicated: (1) Hipot + Functional tests merged into a SINGLE module; (2) Power connection separated from Control/IO - hipot uses only power connections, functional uses power + control; (3) Semi-automated product-to-pallet connection (busbars/needles/pogo - method TBD by supplier), connection movement &amp; fixturing by operator; (4) Visual inspection limited to verifying the HMI is working correctly. Test specification + 3D CAD sent. Medium Drives scope (higher power/current/size) to be sent this week.</t>
+          <t>Fulda, Germany (Edgar Vöhringer). INBOUND contact. Meeting held 24/06/2026. Scope changes communicated: (1) Hipot + Functional tests merged into a SINGLE module; (2) Power connection separated from Control/IO - hipot uses only power connections, functional uses power + control; (3) Semi-automated product-to-pallet connection (busbars/needles/pogo - method TBD by supplier), connection movement &amp; fixturing by operator; (4) Visual inspection limited to verifying the HMI is working correctly. Test specification + 3D CAD sent. Medium Drives scope (higher power/current/size) to be sent this week. FFT replied with 6 technical questions (HMI/visual inspection scope, serial number &amp; MAC source, Modbus comms documentation, fan speed parameter, motor test load, 3D CAD) - WEG answers drafted, pending send.</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Waiting for quotation (after Jul 4th holiday). WEG to send: CAD/connector drawing of product</t>
+          <t>Waiting for quotation (after Jul 4th holiday). WEG to send: CAD/connector drawing of product. Send updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1492,12 +1492,12 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Waiting for quotation. Send: test spec + assembly scope (Alissonn). Provide WEG invitation letter for visa when needed.</t>
+          <t>Quote received. Meeting scheduled to discuss the quote and negotiate price reduction. WEG to send: test spec + assembly scope (Alissonn) + WEG invitation letter for visa when needed. Send updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Part of Dual Group (acquired 2023). HQ Munich. 4 China factories (Suzhou, Tianjin, Kunshan, Xian). ~EUR 200M revenue China. BEST reference: inverter EOL test + PCB/IGBT assembly. WEG PLC: never used - checking. Team Soft (C#) available.</t>
+          <t>Part of Dual Group (acquired 2023). HQ Munich. 4 China factories (Suzhou, Tianjin, Kunshan, Xian). ~EUR 200M revenue China. BEST reference: inverter EOL test + PCB/IGBT assembly. WEG PLC: never used - checking. Team Soft (C#) available. Meeting scheduled (date TBC) to review pricing.</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Waiting for quotation (~next week after holiday). WEG to send: product images + test specification</t>
+          <t>Waiting for quotation (~next week after holiday). WEG to send: product images + test specification. Send updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Record MASMEC/BBS pricing meeting dates and FFT Q&A answered
- MASMEC: pricing negotiation meeting held 02/07/2026
- BBS: pricing negotiation meeting scheduled 13/07/2026
- FFT: 6 technical questions answered 02/07/2026 (incl. WEG inverter
  programming guide + product CAD attachments)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XCyDZxfZxZ3SBQAJkRpEXx
</commit_message>
<xml_diff>
--- a/SUPPLIERS/SUPPLIERS.xlsx
+++ b/SUPPLIERS/SUPPLIERS.xlsx
@@ -991,12 +991,12 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Quote C610222-1 received. Meeting scheduled to discuss the quote and negotiate price reduction. WEG to send: test prescription per module + confirm WEG PLC (not Siemens). Send updated Small-line scope + Medium-line scope (to quote).</t>
+          <t>Quote C610222-1 received. Pricing meeting held 02/07/2026 to negotiate a reduction. WEG to send: test prescription per module + confirm WEG PLC (not Siemens). Send updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Bari, Italy. Direct experience testing automotive inverters (hipot, functional, load). Bosch Rexroth TS2 conveyor. Brazil installs. All machines made in Italy. Digital twin w/ Plant Simulation. Meeting scheduled (date TBC) to review pricing.</t>
+          <t>Bari, Italy. Direct experience testing automotive inverters (hipot, functional, load). Bosch Rexroth TS2 conveyor. Brazil installs. All machines made in Italy. Digital twin w/ Plant Simulation. Pricing negotiation meeting held 02/07/2026.</t>
         </is>
       </c>
     </row>
@@ -1153,12 +1153,12 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>WEG to answer FFT's 6 technical questions and send the WEG inverter programming reference doc + product CAD. Send updated Small-line scope + Medium-line scope (to quote).</t>
+          <t>FFT's 6 technical questions answered (02/07/2026), including attachments (WEG inverter programming guide + product CAD). Send updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Fulda, Germany (Edgar Vöhringer). INBOUND contact. Meeting held 24/06/2026. Scope changes communicated: (1) Hipot + Functional tests merged into a SINGLE module; (2) Power connection separated from Control/IO - hipot uses only power connections, functional uses power + control; (3) Semi-automated product-to-pallet connection (busbars/needles/pogo - method TBD by supplier), connection movement &amp; fixturing by operator; (4) Visual inspection limited to verifying the HMI is working correctly. Test specification + 3D CAD sent. Medium Drives scope (higher power/current/size) to be sent this week. FFT replied with 6 technical questions (HMI/visual inspection scope, serial number &amp; MAC source, Modbus comms documentation, fan speed parameter, motor test load, 3D CAD) - WEG answers drafted, pending send.</t>
+          <t>Fulda, Germany (Edgar Vöhringer). INBOUND contact. Meeting held 24/06/2026. Scope changes communicated: (1) Hipot + Functional tests merged into a SINGLE module; (2) Power connection separated from Control/IO - hipot uses only power connections, functional uses power + control; (3) Semi-automated product-to-pallet connection (busbars/needles/pogo - method TBD by supplier), connection movement &amp; fixturing by operator; (4) Visual inspection limited to verifying the HMI is working correctly. Test specification + 3D CAD sent. Medium Drives scope (higher power/current/size) to be sent this week. FFT replied with 6 technical questions (HMI/visual inspection scope, serial number &amp; MAC source, Modbus comms documentation, fan speed parameter, motor test load, 3D CAD) - answered by WEG on 02/07/2026.</t>
         </is>
       </c>
     </row>
@@ -1492,12 +1492,12 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Quote received. Meeting scheduled to discuss the quote and negotiate price reduction. WEG to send: test spec + assembly scope (Alissonn) + WEG invitation letter for visa when needed. Send updated Small-line scope + Medium-line scope (to quote).</t>
+          <t>Quote received. Pricing meeting scheduled for 13/07/2026 to negotiate a reduction. WEG to send: test spec + assembly scope (Alissonn) + WEG invitation letter for visa when needed. Send updated Small-line scope + Medium-line scope (to quote).</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Part of Dual Group (acquired 2023). HQ Munich. 4 China factories (Suzhou, Tianjin, Kunshan, Xian). ~EUR 200M revenue China. BEST reference: inverter EOL test + PCB/IGBT assembly. WEG PLC: never used - checking. Team Soft (C#) available. Meeting scheduled (date TBC) to review pricing.</t>
+          <t>Part of Dual Group (acquired 2023). HQ Munich. 4 China factories (Suzhou, Tianjin, Kunshan, Xian). ~EUR 200M revenue China. BEST reference: inverter EOL test + PCB/IGBT assembly. WEG PLC: never used - checking. Team Soft (C#) available. Pricing negotiation meeting scheduled for 13/07/2026.</t>
         </is>
       </c>
     </row>

</xml_diff>